<commit_message>
Loading page while load scene
Loading page while load scene
</commit_message>
<xml_diff>
--- a/ConfigExporter/xlsx/ui_page.xlsx
+++ b/ConfigExporter/xlsx/ui_page.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\WeiqiXN\ConfigExporter\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7F412D-B5CB-4B99-A9EB-B499538555AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A6050C0-9817-44F2-8FE5-359C81BEA94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6825" yWindow="6465" windowWidth="29205" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5235" yWindow="2370" windowWidth="29205" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ui_page" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -68,6 +68,22 @@
   </si>
   <si>
     <t>#require#enum(General,Header,Loading,TopMost)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>isLoadAsync</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否异步加载</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>boolean</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>#require</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -430,15 +446,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.625" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.25" style="1" customWidth="1"/>
     <col min="3" max="3" width="23.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.25" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -448,8 +465,11 @@
       <c r="C1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -459,8 +479,11 @@
       <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="D2" s="4" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -470,8 +493,11 @@
       <c r="C3" s="4" t="s">
         <v>1</v>
       </c>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" s="6" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -481,14 +507,20 @@
       <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4" t="s">
         <v>9</v>
+      </c>
+      <c r="D5" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enter game chess board selection
Enter game chess board selection
</commit_message>
<xml_diff>
--- a/ConfigExporter/xlsx/ui_page.xlsx
+++ b/ConfigExporter/xlsx/ui_page.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project\WeiqiXN\ConfigExporter\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\WeiqiXN\ConfigExporter\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E9E75F-92A5-4497-AD8A-CCBC4FF74988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB807448-B27B-4F70-9721-F1A53FBE9C24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2715" windowWidth="29205" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8115" yWindow="5535" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ui_page" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -136,6 +136,14 @@
   </si>
   <si>
     <t>Header</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DuelSetupPopup</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对弈设置弹窗</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -498,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.625" style="1" customWidth="1"/>
@@ -645,18 +653,35 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4" t="b">
+      <c r="D10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="4" t="b">
+      <c r="E10" s="4" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>